<commit_message>
N-PORT Security: matching rules declared, Mapping Documents, quality measured
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XffcaJSmoXmrPyZxCeFHRa
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,40 @@
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml defaults.sources[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security.v1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources[1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources[2]</t>
         </is>
       </c>
     </row>
@@ -554,11 +588,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
@@ -594,17 +628,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>name_of_issuer</t>
+          <t>issuer_lei</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>sec.thirteenf.information_table.security.v1</t>
+          <t>sec.nport.security.v1, sec.nport.security_isin.v1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>sec.thirteenf.information_table.security.v1</t>
+          <t>sec.nport.security.v1</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -621,25 +655,52 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>name_of_issuer</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>sec.thirteenf.information_table.security.v1, sec.nport.security.v1, sec.nport.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>sec.thirteenf.information_table.security.v1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
           <t>title_of_class</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>sec.thirteenf.information_table.security.v1, sec.nport.security.v1, sec.nport.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>sec.thirteenf.information_table.security.v1</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Kind default</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml defaults.sources</t>
         </is>
@@ -722,11 +783,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -812,6 +873,120 @@
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml rules[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>nport-security-cusip</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15.1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security.v1</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>The record's CUSIP is the one a Company holds; and Exactly one Company holds that CUSIP, or none</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml rules[1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>nport-security-isin</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15.1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security.v1</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>The record's ISIN is the one a Company holds; and Exactly one Company holds that ISIN, or none</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml rules[2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>nport-isin-security-isin</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15.1</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>The record's ISIN is the one a Company holds; and Exactly one Company holds that ISIN, or none</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml rules[3]</t>
         </is>
       </c>
     </row>
@@ -873,7 +1048,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -891,7 +1066,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -909,7 +1084,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ticket 80: the openfigi source and its Security matching rules (declared)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199JiQoZJ5my5vrS5tW3FQH
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -574,6 +574,40 @@
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml defaults.sources[2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources[3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources[4]</t>
         </is>
       </c>
     </row>
@@ -783,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -987,6 +1021,82 @@
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml rules[3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>openfigi-security-cusip</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17.1</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>The record's CUSIP is the one a Security holds; and Exactly one Security holds that CUSIP, or none</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>wait</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml rules[4]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>openfigi-security-isin</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17.1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>The record's ISIN is the one a Security holds; and Exactly one Security holds that ISIN, or none</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>wait</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml rules[5]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticket 120: OpenFIGI's Security carries every field, its primary listing's, and every listing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kd1ZT9nNA7gETeQM4V4YtE
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -622,10 +622,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -689,12 +689,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>name_of_issuer</t>
+          <t>market_sector</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1, sec.nport.security.v1, sec.nport.security_isin.v1, sec.thirteenf.information_table.security.v1</t>
+          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -716,25 +716,133 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>name_of_issuer</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1, openfigi.security_isin.v1, sec.nport.security.v1, sec.nport.security_isin.v1, sec.thirteenf.information_table.security.v1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>security_type</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>security_type2</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>share_class_figi</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>title_of_class</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>sec.nport.security.v1, sec.nport.security_isin.v1, sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>sec.nport.security.v1</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Kind default</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml defaults.sources</t>
         </is>

</xml_diff>

<commit_message>
Ticket 120: one Security record per Security from N-PORT (sec.nport.security.v2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kd1ZT9nNA7gETeQM4V4YtE
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -568,7 +568,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v1</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -585,29 +585,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security_isin.v1</t>
+          <t>sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml defaults.sources[3]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>sec.thirteenf.information_table.security.v1</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/security.yaml defaults.sources[4]</t>
         </is>
       </c>
     </row>
@@ -667,12 +650,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v1, sec.nport.security_isin.v1</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v1</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -721,7 +704,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1, sec.nport.security.v1, sec.nport.security_isin.v1, sec.thirteenf.information_table.security.v1</t>
+          <t>openfigi.security.v1, openfigi.security_isin.v1, sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -829,12 +812,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v1, sec.nport.security_isin.v1, sec.thirteenf.information_table.security.v1</t>
+          <t>sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v1</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -925,11 +908,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -1031,12 +1014,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-20.1</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v1</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -1069,12 +1052,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-20.1</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v1</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -1102,28 +1085,28 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>nport-isin-security-isin</t>
+          <t>openfigi-security-cusip</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-17.1</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security_isin.v1</t>
+          <t>openfigi.security.v1</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>The record's ISIN is the one a Security holds; and Exactly one Security holds that ISIN, or none</t>
+          <t>The record's CUSIP is the one a Security holds; and Exactly one Security holds that CUSIP, or none</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>mint</t>
+          <t>wait</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1140,7 +1123,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>openfigi-security-cusip</t>
+          <t>openfigi-security-isin</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1150,13 +1133,13 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1</t>
+          <t>openfigi.security_isin.v1</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>The record's CUSIP is the one a Security holds; and Exactly one Security holds that CUSIP, or none</t>
+          <t>The record's ISIN is the one a Security holds; and Exactly one Security holds that ISIN, or none</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1167,44 +1150,6 @@
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml rules[4]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>openfigi-security-isin</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17.1</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>openfigi.security_isin.v1</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>The record's ISIN is the one a Security holds; and Exactly one Security holds that ISIN, or none</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>wait</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/security.yaml rules[5]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticket 129: the filed issuer LEI leaves the Security for silver; skill rules
Review of every MDM field against the data-onboarding map rules (operator,
2026-10-22). Fix 1: `issuer_lei` is no longer an N-PORT Security field (an LEI
identifies a Company; the Security reaches its issuer by ISSUED_BY); the LEI
each fund filed is a column of the silver holding row. MAPPING.xlsx and
security.xlsx regenerated.

Skills, with the operator's ruling "date that changes usually should not be
in MDM unless it adds meaning to the entity or turn on or off":
data-onboarding (map "Fields") and refining-rules (which target a field
belongs to; a field change regenerates both workbooks). Ticket 129 records
the review; fix 2 (the GLEIF dates) is engine work and follows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YGQ3FjYgHS7jgMe6eLB7Z3
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -645,17 +645,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>issuer_lei</t>
+          <t>market_sector</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v2</t>
+          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v2</t>
+          <t>openfigi.security.v1</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -672,12 +672,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>market_sector</t>
+          <t>name_of_issuer</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
+          <t>openfigi.security.v1, openfigi.security_isin.v1, sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -699,12 +699,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>name_of_issuer</t>
+          <t>security_type</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1, sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
+          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -726,7 +726,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>security_type</t>
+          <t>security_type2</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -753,7 +753,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>security_type2</t>
+          <t>share_class_figi</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -780,17 +780,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>share_class_figi</t>
+          <t>title_of_class</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
+          <t>sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -799,33 +799,6 @@
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/security.yaml defaults.sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>title_of_class</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>sec.nport.security.v2</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Kind default</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml defaults.sources</t>
         </is>

</xml_diff>

<commit_message>
Ticket 129, fix 4: share_class_figi is a cross-reference only
Operator: "Fix 4". The two OpenFIGI Security contracts no longer map it as a
field too; MAPPING.xlsx and security.xlsx regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YGQ3FjYgHS7jgMe6eLB7Z3
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -605,10 +605,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -753,17 +753,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>share_class_figi</t>
+          <t>title_of_class</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
+          <t>sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -772,33 +772,6 @@
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/security.yaml defaults.sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>title_of_class</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>sec.nport.security.v2</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Kind default</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml defaults.sources</t>
         </is>

</xml_diff>

<commit_message>
Ticket 130: a Security's share class from its filed titles
The Security gets `share_class`, one letter, from "CL", "CLASS" or "CLS"
then a letter in the filed titles (13F; N-PORT equity holdings only).
Filers that name two letters give none, and a flag-only quality check
lists the Security. Workbooks regenerated; skills learn the patterns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YGQ3FjYgHS7jgMe6eLB7Z3
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -753,25 +753,52 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>share_class</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security.v2</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>title_of_class</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>sec.nport.security.v2</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Kind default</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml defaults.sources</t>
         </is>

</xml_diff>

<commit_message>
Give the OpenFIGI ISIN contract its own source code so it can be activated.
company-on already held openfigi.security_isin.v1. The contract now also issues a CUSIP, and that identity cannot change on the registered code. The dataset is openfigi.security_isin.v2. The proved Securities source is the one a run will use.
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>security-2026-10-23.openfigi-first</t>
+          <t>security-2026-10-24.isin-source-code</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security_isin.v1</t>
+          <t>openfigi.security_isin.v2</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
+          <t>openfigi.security.v1, openfigi.security_isin.v2</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1, sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
+          <t>openfigi.security.v1, openfigi.security_isin.v2, sec.nport.security.v2, sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
+          <t>openfigi.security.v1, openfigi.security_isin.v2</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v1, openfigi.security_isin.v1</t>
+          <t>openfigi.security.v1, openfigi.security_isin.v2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1101,12 +1101,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security_isin.v1</t>
+          <t>openfigi.security_isin.v2</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security_isin.v1</t>
+          <t>openfigi.security_isin.v2</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Ticket 138 part A2a: FIGIs reaching two Securities merge them (#1182)
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>security-2026-10-25.one-openfigi-load</t>
+          <t>security-2026-10-26.figi-merges-securities</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25.1</t>
+          <t>2026-10-26.1</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ticket 138 Design 5: a FIGI 13F files finds its Security, lookup only
The operator, 2026-10-26 14:42 ET, "Lookup only (Recommended)": a FIGI a
filer states finds the Security OpenFIGI gave it to; it never becomes that
Security's identifier and never merges; the CUSIP wins a conflict.

- Engine: a matching rule on an identifier its record's source does not
  issue reads the record's cross-reference when the record carries no such
  identifier. It finds the holders; the value is never minted (the source
  issues nothing), so no projection, holder or index reads it as held.
- Activation: only the identifier's issuing source may merge by it.
- 13F: `thirteenf-security-figi` ("Filed FIGI finds its Security") and
  `security-cusip` 2026-10-26.1 ("Filed CUSIP wins over a filed FIGI").
  The 2026-10-14.1 switch-on ends; both wait for the operator's switch-on.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASjL6aq7noeTrLkwhheAnB
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>security-2026-10-26.filed-cusip-binds-first</t>
+          <t>security-2026-10-26.filed-figi-finds</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -932,7 +932,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14.1</t>
+          <t>2026-10-26.1</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -965,28 +965,28 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>nport-security-cusip</t>
+          <t>thirteenf-security-figi</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26.2</t>
+          <t>2026-10-26.1</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>sec.nport.security.v2</t>
+          <t>sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>The record's CUSIP is the one a Security holds; and Exactly one Security holds that CUSIP, or none</t>
+          <t>The record's FIGI is the one a Security holds; and Exactly one Security holds that FIGI, or none</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>mint</t>
+          <t>wait</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1003,12 +1003,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>nport-security-isin</t>
+          <t>nport-security-cusip</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26.1</t>
+          <t>2026-10-26.2</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1019,7 +1019,7 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>The record's ISIN is the one a Security holds; and Exactly one Security holds that ISIN, or none</t>
+          <t>The record's CUSIP is the one a Security holds; and Exactly one Security holds that CUSIP, or none</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1041,23 +1041,23 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>openfigi-security-cusip</t>
+          <t>nport-security-isin</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25.1</t>
+          <t>2026-10-26.1</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v3</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>The record's CUSIP is the one a Security holds; and Exactly one Security holds that CUSIP, or none</t>
+          <t>The record's ISIN is the one a Security holds; and Exactly one Security holds that ISIN, or none</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>openfigi-security-isin</t>
+          <t>openfigi-security-cusip</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1095,7 +1095,7 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>The record's ISIN is the one a Security holds; and Exactly one Security holds that ISIN, or none</t>
+          <t>The record's CUSIP is the one a Security holds; and Exactly one Security holds that CUSIP, or none</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>openfigi-security-figi</t>
+          <t>openfigi-security-isin</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26.1</t>
+          <t>2026-10-25.1</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1133,17 +1133,55 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>The record's ISIN is the one a Security holds; and Exactly one Security holds that ISIN, or none</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml rules[5]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>openfigi-security-figi</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26.1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v3</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>The record's FIGI is the one a Security holds; and Exactly one Security holds that FIGI, or none</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>mint</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/security.yaml rules[5]</t>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml rules[6]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticket 138: switch on the 13F filed FIGI rule; put/call FIGIs set aside
Operator, 2026-10-27: "On, set aside put/call (Recommended)".

- security-cusip 2026-10-27.1 ("13F CUSIP binds first", on_conflict: first)
  and thirteenf-security-figi switched on: a 13F CUSIP no Security holds
  joins the Security holding its filed FIGI; a held CUSIP stays put.
- The 13F source extract reads a FIGI only from a row with no put or call
  (97 of 10,681 CUSIPs with a filed FIGI lose it, 4 keep another).
- Limited test counts in research/138_13f_figi_limited_test.json.
- data-operations skill: long runs under caffeinate -i (this Mac sleeps
  after one idle minute and freezes Docker).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASjL6aq7noeTrLkwhheAnB
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>security-2026-10-26.filed-figi-finds</t>
+          <t>security-2026-10-27.filed-figi-on</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14.1</t>
+          <t>2026-10-27.1</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ticket 138: N-PORT's six Security facts on the master, by most-filed value
A reduction gains `mode: most`: per key, the member the most rows file; a
tie keeps none; a row filing none votes for none. N-PORT's Security tables
carry asset category, issuer type, investment country, currency, restricted
and derivative category; reduce, combine and record take each Security's
most-filed value into the Dataset Contract (adapter v4). The holding's silver
row drops its nine copies of master fields (one system of record, ticket 143).
Off until a limited test and the operator's switch-on. Ticket 132's PR line
ticked (#1196).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASjL6aq7noeTrLkwhheAnB
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/security.xlsx
+++ b/rules/merge/kinds/security.xlsx
@@ -588,10 +588,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -628,17 +628,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>market_sector</t>
+          <t>asset_category</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v3</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v3</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -655,17 +655,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>name_of_issuer</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v3, sec.thirteenf.information_table.security.v1, sec.nport.security.v2</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v3</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -682,17 +682,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>security_type</t>
+          <t>derivative_category</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v3</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v3</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -709,17 +709,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>security_type2</t>
+          <t>investment_country</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v3</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>openfigi.security.v3</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -736,17 +736,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>share_class</t>
+          <t>issuer_type</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>sec.thirteenf.information_table.security.v1, sec.nport.security.v2</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>sec.thirteenf.information_table.security.v1</t>
+          <t>sec.nport.security.v2</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -763,25 +763,187 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>market_sector</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v3</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v3</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>name_of_issuer</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v3, sec.thirteenf.information_table.security.v1, sec.nport.security.v2</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v3</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>restricted</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security.v2</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security.v2</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>security_type</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v3</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v3</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>security_type2</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v3</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>openfigi.security.v3</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>share_class</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>sec.thirteenf.information_table.security.v1, sec.nport.security.v2</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>sec.thirteenf.information_table.security.v1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/security.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>title_of_class</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>sec.thirteenf.information_table.security.v1, sec.nport.security.v2</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>sec.thirteenf.information_table.security.v1</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Kind default</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/security.yaml defaults.sources</t>
         </is>

</xml_diff>